<commit_message>
report: v2 Rules_Report states the RELREC key of a forward-RELREC rule (OD-9, FU-4 (a)) + XLSX column
OSS port of cumba-corej 38b4fe9, byte-identical (PLAN-merge-followups item 4,
FU-4 (a)): a rule with a forward RELREC entry carries the v2-only relrec_key
(SDTM / SEND key, the spelled-out inference under UNKNOWN), derived from the
conformance's Standard — the run standard's name, exactly the merge's
mergeStandardOf; v1 stays frozen (withoutV2OnlyRuleKeys); the XLSX v2 rule
sheet gains the RELREC Key column; golden.xlsx regenerated (one resolved-value
difference, Rules Report!J1).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014gSewu81vXFCpEaeXK9hy8
</commit_message>
<xml_diff>
--- a/lib/cumba-oss-corej-report-xlsx/src/test/resources/report/golden.xlsx
+++ b/lib/cumba-oss-corej-report-xlsx/src/test/resources/report/golden.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="98">
   <si>
     <t>CORE-ID</t>
   </si>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>Errored</t>
+  </si>
+  <si>
+    <t>RELREC Key</t>
   </si>
   <si>
     <t>CG0001</t>
@@ -2426,7 +2429,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I197"/>
+  <dimension ref="A1:J197"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="4" width="19.109375"/>
@@ -2438,6 +2441,7 @@
     <col min="7" max="7" bestFit="true" customWidth="true" width="12.0"/>
     <col min="8" max="8" width="12.0" customWidth="true"/>
     <col min="9" max="9" width="12.0" customWidth="true"/>
+    <col min="10" max="10" width="48.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2468,6 +2472,9 @@
       <c r="I1" s="10" t="s">
         <v>84</v>
       </c>
+      <c r="J1" s="10" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
@@ -2477,18 +2484,19 @@
         <v>72</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D2" s="15"/>
       <c r="E2" s="16" t="s">
         <v>65</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
       <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -2498,41 +2506,43 @@
         <v>76</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E3" s="16" t="s">
         <v>68</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
       <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
     </row>
     <row r="4" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>72</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D4" s="15"/>
       <c r="E4" s="16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
       <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
     </row>
     <row r="5" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
@@ -3146,24 +3156,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B1" t="s" s="0">
         <v>7</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>